<commit_message>
re-run proccessing to improve CH4 data
</commit_message>
<xml_diff>
--- a/data/sampling/ghg/ghg_data.xlsx
+++ b/data/sampling/ghg/ghg_data.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/ECM/alhic1901_deep_layering/github/data/sampling/ghg/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/ghg/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D46A63B8-E5CD-C646-B5E6-3DB60EEA6DA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F76373-1B2E-CE46-8727-9283B1613FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="180" yWindow="-21640" windowWidth="29220" windowHeight="18880" xr2:uid="{5D78C863-DB51-414A-8C70-78F5C24BA3CE}"/>
+    <workbookView xWindow="-7860" yWindow="-20820" windowWidth="29160" windowHeight="18980" xr2:uid="{5D78C863-DB51-414A-8C70-78F5C24BA3CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="47">
   <si>
     <t>section</t>
   </si>
@@ -182,6 +183,24 @@
   </si>
   <si>
     <t>dxs</t>
+  </si>
+  <si>
+    <t>left_topdepth</t>
+  </si>
+  <si>
+    <t>right_topdepth</t>
+  </si>
+  <si>
+    <t>top_left_depth</t>
+  </si>
+  <si>
+    <t>top_right_depth</t>
+  </si>
+  <si>
+    <t>bottom_left_depth</t>
+  </si>
+  <si>
+    <t>bottom_right_depth</t>
   </si>
 </sst>
 </file>
@@ -191,7 +210,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -204,6 +223,18 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -226,10 +257,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -564,10 +597,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC37B97-9650-DA43-B790-3970A5ED3209}">
-  <dimension ref="A1:K41"/>
+  <dimension ref="A1:O41"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="7" max="7" width="14.33203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -584,25 +622,37 @@
         <v>6</v>
       </c>
       <c r="F1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="K1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="L1" t="s">
         <v>3</v>
       </c>
-      <c r="I1" t="s">
+      <c r="M1" t="s">
         <v>38</v>
       </c>
-      <c r="J1" t="s">
+      <c r="N1" t="s">
         <v>39</v>
       </c>
-      <c r="K1" t="s">
+      <c r="O1" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -618,14 +668,26 @@
       <c r="E2">
         <v>155.08625000000001</v>
       </c>
+      <c r="F2">
+        <v>155.08849999999998</v>
+      </c>
       <c r="G2">
+        <v>155.07749999999999</v>
+      </c>
+      <c r="H2">
+        <v>155.10249999999999</v>
+      </c>
+      <c r="I2">
+        <v>155.1215</v>
+      </c>
+      <c r="K2">
         <v>513.39643590000003</v>
       </c>
-      <c r="H2">
+      <c r="L2">
         <v>0.100997292</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -641,14 +703,26 @@
       <c r="E3">
         <v>155.11250000000001</v>
       </c>
+      <c r="F3">
+        <v>155.10249999999999</v>
+      </c>
       <c r="G3">
+        <v>155.1215</v>
+      </c>
+      <c r="H3">
+        <v>155.1275</v>
+      </c>
+      <c r="I3">
+        <v>155.1525</v>
+      </c>
+      <c r="K3">
         <v>521.20168609999996</v>
       </c>
-      <c r="H3">
+      <c r="L3">
         <v>9.7894287999999996E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -664,14 +738,26 @@
       <c r="E4">
         <v>155.13749999999999</v>
       </c>
+      <c r="F4">
+        <v>155.1275</v>
+      </c>
       <c r="G4">
+        <v>155.1525</v>
+      </c>
+      <c r="H4">
+        <v>155.1575</v>
+      </c>
+      <c r="I4">
+        <v>155.1765</v>
+      </c>
+      <c r="K4">
         <v>566.79918099999998</v>
       </c>
-      <c r="H4">
+      <c r="L4">
         <v>9.3101737000000004E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -687,14 +773,26 @@
       <c r="E5">
         <v>155.16249999999999</v>
       </c>
+      <c r="F5">
+        <v>155.1575</v>
+      </c>
       <c r="G5">
+        <v>155.1765</v>
+      </c>
+      <c r="H5">
+        <v>155.17949999999999</v>
+      </c>
+      <c r="I5">
+        <v>155.20249999999999</v>
+      </c>
+      <c r="K5">
         <v>575.73996339999997</v>
       </c>
-      <c r="H5">
+      <c r="L5">
         <v>9.6401944000000003E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -710,14 +808,26 @@
       <c r="E6">
         <v>155.1875</v>
       </c>
+      <c r="F6">
+        <v>155.17949999999999</v>
+      </c>
       <c r="G6">
+        <v>155.20249999999999</v>
+      </c>
+      <c r="H6">
+        <v>155.2045</v>
+      </c>
+      <c r="I6">
+        <v>155.22749999999999</v>
+      </c>
+      <c r="K6">
         <v>593.48608549999994</v>
       </c>
-      <c r="H6">
+      <c r="L6">
         <v>0.100555226</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -733,14 +843,26 @@
       <c r="E7">
         <v>155.21375</v>
       </c>
+      <c r="F7">
+        <v>155.2045</v>
+      </c>
       <c r="G7">
+        <v>155.22749999999999</v>
+      </c>
+      <c r="H7">
+        <v>155.2405</v>
+      </c>
+      <c r="I7">
+        <v>155.25649999999999</v>
+      </c>
+      <c r="K7">
         <v>618.58037349999995</v>
       </c>
-      <c r="H7">
+      <c r="L7">
         <v>9.6052947999999999E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -756,14 +878,26 @@
       <c r="E8">
         <v>155.24875</v>
       </c>
+      <c r="F8">
+        <v>155.2405</v>
+      </c>
       <c r="G8">
+        <v>155.25649999999999</v>
+      </c>
+      <c r="H8">
+        <v>155.2645</v>
+      </c>
+      <c r="I8">
+        <v>155.28749999999999</v>
+      </c>
+      <c r="K8">
         <v>627.77715360000002</v>
       </c>
-      <c r="H8">
+      <c r="L8">
         <v>9.6107177000000002E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -779,14 +913,26 @@
       <c r="E9">
         <v>155.2825</v>
       </c>
+      <c r="F9">
+        <v>155.2645</v>
+      </c>
       <c r="G9">
+        <v>155.28749999999999</v>
+      </c>
+      <c r="H9">
+        <v>155.2895</v>
+      </c>
+      <c r="I9">
+        <v>155.3125</v>
+      </c>
+      <c r="K9">
         <v>578.25503690000005</v>
       </c>
-      <c r="H9">
+      <c r="L9">
         <v>9.9159223000000005E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -802,14 +948,26 @@
       <c r="E10">
         <v>155.3075</v>
       </c>
+      <c r="F10">
+        <v>155.2895</v>
+      </c>
       <c r="G10">
+        <v>155.3125</v>
+      </c>
+      <c r="H10">
+        <v>155.33249999999998</v>
+      </c>
+      <c r="I10">
+        <v>155.3175</v>
+      </c>
+      <c r="K10">
         <v>572.04765689999999</v>
       </c>
-      <c r="H10">
+      <c r="L10">
         <v>8.5164080000000003E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -825,11 +983,11 @@
       <c r="E11">
         <v>155.08125000000001</v>
       </c>
-      <c r="F11">
+      <c r="J11">
         <v>646</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -845,11 +1003,11 @@
       <c r="E12">
         <v>155.10249999999999</v>
       </c>
-      <c r="F12">
+      <c r="J12">
         <v>751</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -865,11 +1023,11 @@
       <c r="E13">
         <v>155.12625</v>
       </c>
-      <c r="F13">
+      <c r="J13">
         <v>799</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -885,11 +1043,11 @@
       <c r="E14">
         <v>155.15125</v>
       </c>
-      <c r="F14">
+      <c r="J14">
         <v>822</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -905,11 +1063,11 @@
       <c r="E15">
         <v>155.17250000000001</v>
       </c>
-      <c r="F15">
+      <c r="J15">
         <v>818.9</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -925,11 +1083,11 @@
       <c r="E16">
         <v>155.1925</v>
       </c>
-      <c r="F16">
+      <c r="J16">
         <v>793.46</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>9</v>
       </c>
@@ -945,11 +1103,11 @@
       <c r="E17">
         <v>155.21250000000001</v>
       </c>
-      <c r="F17">
+      <c r="J17">
         <v>773.09</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>9</v>
       </c>
@@ -965,11 +1123,11 @@
       <c r="E18">
         <v>155.24</v>
       </c>
-      <c r="F18">
+      <c r="J18">
         <v>741.4</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>9</v>
       </c>
@@ -985,11 +1143,11 @@
       <c r="E19">
         <v>155.26750000000001</v>
       </c>
-      <c r="F19">
+      <c r="J19">
         <v>731.26</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>9</v>
       </c>
@@ -1005,11 +1163,11 @@
       <c r="E20">
         <v>155.28749999999999</v>
       </c>
-      <c r="F20">
+      <c r="J20">
         <v>727.65</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>9</v>
       </c>
@@ -1025,11 +1183,11 @@
       <c r="E21">
         <v>155.3075</v>
       </c>
-      <c r="F21">
+      <c r="J21">
         <v>740.8</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>9</v>
       </c>
@@ -1045,11 +1203,11 @@
       <c r="E22">
         <v>155.32374999999999</v>
       </c>
-      <c r="F22">
+      <c r="J22">
         <v>769.28</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -1066,11 +1224,11 @@
       <c r="E23">
         <v>156.80150000000003</v>
       </c>
-      <c r="F23" s="1">
+      <c r="J23" s="1">
         <v>929.65326090001497</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -1086,11 +1244,11 @@
       <c r="E24">
         <v>156.82700000000003</v>
       </c>
-      <c r="F24" s="1">
+      <c r="J24" s="1">
         <v>930.44694399046705</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -1106,11 +1264,11 @@
       <c r="E25">
         <v>156.85100000000003</v>
       </c>
-      <c r="F25" s="1">
+      <c r="J25" s="1">
         <v>914.58605951339928</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>11</v>
       </c>
@@ -1126,11 +1284,11 @@
       <c r="E26">
         <v>156.875</v>
       </c>
-      <c r="F26" s="1">
+      <c r="J26" s="1">
         <v>905.49576901251248</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -1146,11 +1304,11 @@
       <c r="E27">
         <v>156.90650000000002</v>
       </c>
-      <c r="F27" s="1">
+      <c r="J27" s="1">
         <v>913.69238545090184</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -1166,11 +1324,11 @@
       <c r="E28">
         <v>156.92700000000002</v>
       </c>
-      <c r="F28" s="1">
+      <c r="J28" s="1">
         <v>896.00585988279863</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -1186,11 +1344,11 @@
       <c r="E29">
         <v>156.95200000000003</v>
       </c>
-      <c r="F29" s="1">
+      <c r="J29" s="1">
         <v>805.47451233658978</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -1206,11 +1364,11 @@
       <c r="E30">
         <v>156.97250000000003</v>
       </c>
-      <c r="F30" s="1">
+      <c r="J30" s="1">
         <v>751.76754234764746</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -1226,11 +1384,11 @@
       <c r="E31">
         <v>157.00200000000001</v>
       </c>
-      <c r="F31" s="1">
+      <c r="J31" s="1">
         <v>687.20098795460331</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>11</v>
       </c>
@@ -1246,11 +1404,11 @@
       <c r="E32">
         <v>157.0265</v>
       </c>
-      <c r="F32" s="1">
+      <c r="J32" s="1">
         <v>711.56288936566284</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -1266,11 +1424,11 @@
       <c r="E33">
         <v>157.04400000000001</v>
       </c>
-      <c r="F33" s="1">
+      <c r="J33" s="1">
         <v>743.06784778646261</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>11</v>
       </c>
@@ -1287,23 +1445,23 @@
         <f>(C34+D34)/2</f>
         <v>156.81400000000002</v>
       </c>
-      <c r="G34" s="1">
+      <c r="K34" s="1">
         <v>567.53034109412488</v>
       </c>
-      <c r="H34" s="2">
+      <c r="L34" s="2">
         <v>9.305033515712835E-2</v>
       </c>
-      <c r="I34">
+      <c r="M34">
         <v>-35.9</v>
       </c>
-      <c r="J34">
+      <c r="N34">
         <v>-285.98</v>
       </c>
-      <c r="K34">
+      <c r="O34">
         <v>1.18</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>11</v>
       </c>
@@ -1320,23 +1478,23 @@
         <f t="shared" ref="E35:E41" si="0">(C35+D35)/2</f>
         <v>156.84450000000001</v>
       </c>
-      <c r="G35" s="1">
+      <c r="K35" s="1">
         <v>541.7870376085981</v>
       </c>
-      <c r="H35" s="2">
+      <c r="L35" s="2">
         <v>0.10142986414336898</v>
       </c>
-      <c r="I35">
+      <c r="M35">
         <v>-35.270000000000003</v>
       </c>
-      <c r="J35">
+      <c r="N35">
         <v>-279.61</v>
       </c>
-      <c r="K35">
+      <c r="O35">
         <v>2.56</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>11</v>
       </c>
@@ -1353,23 +1511,23 @@
         <f t="shared" si="0"/>
         <v>156.87450000000001</v>
       </c>
-      <c r="G36" s="1">
+      <c r="K36" s="1">
         <v>544.69363399218207</v>
       </c>
-      <c r="H36" s="2">
+      <c r="L36" s="2">
         <v>0.10408078150319912</v>
       </c>
-      <c r="I36">
+      <c r="M36">
         <v>-35.32</v>
       </c>
-      <c r="J36">
+      <c r="N36">
         <v>-279.70999999999998</v>
       </c>
-      <c r="K36">
+      <c r="O36">
         <v>2.86</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -1386,23 +1544,23 @@
         <f t="shared" si="0"/>
         <v>156.90800000000002</v>
       </c>
-      <c r="G37" s="1">
+      <c r="K37" s="1">
         <v>570.64606286429944</v>
       </c>
-      <c r="H37" s="2">
+      <c r="L37" s="2">
         <v>0.10197487540962179</v>
       </c>
-      <c r="I37">
+      <c r="M37">
         <v>-36.15</v>
       </c>
-      <c r="J37">
+      <c r="N37">
         <v>-287.45</v>
       </c>
-      <c r="K37">
+      <c r="O37">
         <v>1.76</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -1410,32 +1568,32 @@
         <v>4</v>
       </c>
       <c r="C38">
-        <v>156.96</v>
+        <v>156.91999999999999</v>
       </c>
       <c r="D38">
         <v>156.94900000000001</v>
       </c>
       <c r="E38">
         <f t="shared" si="0"/>
-        <v>156.9545</v>
-      </c>
-      <c r="G38" s="1">
+        <v>156.93450000000001</v>
+      </c>
+      <c r="K38" s="1">
         <v>554.98770044359424</v>
       </c>
-      <c r="H38" s="2">
+      <c r="L38" s="2">
         <v>8.9376775506879905E-2</v>
       </c>
-      <c r="I38">
+      <c r="M38">
         <v>-36.229999999999997</v>
       </c>
-      <c r="J38">
+      <c r="N38">
         <v>-287.79000000000002</v>
       </c>
-      <c r="K38">
+      <c r="O38">
         <v>2.09</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>11</v>
       </c>
@@ -1452,23 +1610,23 @@
         <f t="shared" si="0"/>
         <v>156.96450000000002</v>
       </c>
-      <c r="G39" s="1">
+      <c r="K39" s="1">
         <v>532.09055041227077</v>
       </c>
-      <c r="H39" s="2">
+      <c r="L39" s="2">
         <v>0.10579916320348218</v>
       </c>
-      <c r="I39">
+      <c r="M39">
         <v>-36.76</v>
       </c>
-      <c r="J39">
+      <c r="N39">
         <v>-293.05</v>
       </c>
-      <c r="K39">
+      <c r="O39">
         <v>1.04</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -1485,23 +1643,23 @@
         <f t="shared" si="0"/>
         <v>156.99450000000002</v>
       </c>
-      <c r="G40" s="1">
+      <c r="K40" s="1">
         <v>529.34462553646142</v>
       </c>
-      <c r="H40" s="2">
+      <c r="L40" s="2">
         <v>9.8586253797180265E-2</v>
       </c>
-      <c r="I40">
+      <c r="M40">
         <v>-36.79</v>
       </c>
-      <c r="J40">
+      <c r="N40">
         <v>-293.38</v>
       </c>
-      <c r="K40">
+      <c r="O40">
         <v>0.97</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>11</v>
       </c>
@@ -1518,19 +1676,19 @@
         <f t="shared" si="0"/>
         <v>157.03300000000002</v>
       </c>
-      <c r="G41" s="1">
+      <c r="K41" s="1">
         <v>564.33435437120465</v>
       </c>
-      <c r="H41" s="2">
+      <c r="L41" s="2">
         <v>0.10389318490035435</v>
       </c>
-      <c r="I41">
+      <c r="M41">
         <v>-36.57</v>
       </c>
-      <c r="J41">
+      <c r="N41">
         <v>-291.25</v>
       </c>
-      <c r="K41">
+      <c r="O41">
         <v>1.33</v>
       </c>
     </row>
@@ -1541,16 +1699,622 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A36881-0611-A543-91F5-CA8955EF1326}">
+  <dimension ref="A1:Q10"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="25.33203125" customWidth="1"/>
+    <col min="9" max="9" width="28.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>43</v>
+      </c>
+      <c r="G1" t="s">
+        <v>44</v>
+      </c>
+      <c r="H1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I1" t="s">
+        <v>46</v>
+      </c>
+      <c r="N1" t="s">
+        <v>43</v>
+      </c>
+      <c r="O1" t="s">
+        <v>44</v>
+      </c>
+      <c r="P1" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2">
+        <v>155.07249999999999</v>
+      </c>
+      <c r="D2">
+        <v>155.1</v>
+      </c>
+      <c r="E2">
+        <v>155.08625000000001</v>
+      </c>
+      <c r="F2">
+        <f>C2-(K2-J2)/200</f>
+        <v>155.078</v>
+      </c>
+      <c r="G2">
+        <f>C2+(K2-J2)/200</f>
+        <v>155.06699999999998</v>
+      </c>
+      <c r="H2">
+        <f>C2-(L2-M2)/200</f>
+        <v>155.08199999999999</v>
+      </c>
+      <c r="I2">
+        <f>D2+(M2-N2)/200</f>
+        <v>154.34905749999999</v>
+      </c>
+      <c r="J2" s="4">
+        <v>1.6</v>
+      </c>
+      <c r="K2" s="4">
+        <v>0.5</v>
+      </c>
+      <c r="L2" s="4">
+        <v>3</v>
+      </c>
+      <c r="M2" s="4">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="N2">
+        <f>$C$2+J2/100</f>
+        <v>155.08849999999998</v>
+      </c>
+      <c r="O2">
+        <f t="shared" ref="O2:R2" si="0">$C$2+K2/100</f>
+        <v>155.07749999999999</v>
+      </c>
+      <c r="P2">
+        <f t="shared" si="0"/>
+        <v>155.10249999999999</v>
+      </c>
+      <c r="Q2">
+        <f t="shared" si="0"/>
+        <v>155.1215</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3">
+        <v>155.1</v>
+      </c>
+      <c r="D3">
+        <v>155.125</v>
+      </c>
+      <c r="E3">
+        <v>155.11250000000001</v>
+      </c>
+      <c r="F3">
+        <f t="shared" ref="F3:F10" si="1">C3-(K3-J3)/200</f>
+        <v>155.09049999999999</v>
+      </c>
+      <c r="G3">
+        <f t="shared" ref="G3:G10" si="2">C3+(K3-J3)/200</f>
+        <v>155.1095</v>
+      </c>
+      <c r="H3">
+        <f t="shared" ref="H3:H10" si="3">C3-(L3-M3)/200</f>
+        <v>155.11249999999998</v>
+      </c>
+      <c r="I3">
+        <f t="shared" ref="I3:I10" si="4">D3+(M3-N3)/200</f>
+        <v>154.3894875</v>
+      </c>
+      <c r="J3" s="4">
+        <v>3</v>
+      </c>
+      <c r="K3" s="4">
+        <v>4.9000000000000004</v>
+      </c>
+      <c r="L3" s="4">
+        <v>5.5</v>
+      </c>
+      <c r="M3" s="4">
+        <v>8</v>
+      </c>
+      <c r="N3">
+        <f t="shared" ref="N3:N10" si="5">$C$2+J3/100</f>
+        <v>155.10249999999999</v>
+      </c>
+      <c r="O3">
+        <f t="shared" ref="O3:O10" si="6">$C$2+K3/100</f>
+        <v>155.1215</v>
+      </c>
+      <c r="P3">
+        <f t="shared" ref="P3:P10" si="7">$C$2+L3/100</f>
+        <v>155.1275</v>
+      </c>
+      <c r="Q3">
+        <f t="shared" ref="Q3:Q10" si="8">$C$2+M3/100</f>
+        <v>155.1525</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4">
+        <v>155.125</v>
+      </c>
+      <c r="D4">
+        <v>155.15</v>
+      </c>
+      <c r="E4">
+        <v>155.13749999999999</v>
+      </c>
+      <c r="F4">
+        <f t="shared" si="1"/>
+        <v>155.11250000000001</v>
+      </c>
+      <c r="G4">
+        <f t="shared" si="2"/>
+        <v>155.13749999999999</v>
+      </c>
+      <c r="H4">
+        <f t="shared" si="3"/>
+        <v>155.1345</v>
+      </c>
+      <c r="I4">
+        <f t="shared" si="4"/>
+        <v>154.42636250000001</v>
+      </c>
+      <c r="J4" s="4">
+        <v>5.5</v>
+      </c>
+      <c r="K4" s="4">
+        <v>8</v>
+      </c>
+      <c r="L4" s="4">
+        <v>8.5</v>
+      </c>
+      <c r="M4" s="4">
+        <v>10.4</v>
+      </c>
+      <c r="N4">
+        <f t="shared" si="5"/>
+        <v>155.1275</v>
+      </c>
+      <c r="O4">
+        <f t="shared" si="6"/>
+        <v>155.1525</v>
+      </c>
+      <c r="P4">
+        <f t="shared" si="7"/>
+        <v>155.1575</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" si="8"/>
+        <v>155.1765</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5">
+        <v>155.15</v>
+      </c>
+      <c r="D5">
+        <v>155.17500000000001</v>
+      </c>
+      <c r="E5">
+        <v>155.16249999999999</v>
+      </c>
+      <c r="F5">
+        <f t="shared" si="1"/>
+        <v>155.1405</v>
+      </c>
+      <c r="G5">
+        <f t="shared" si="2"/>
+        <v>155.15950000000001</v>
+      </c>
+      <c r="H5">
+        <f t="shared" si="3"/>
+        <v>155.16150000000002</v>
+      </c>
+      <c r="I5">
+        <f t="shared" si="4"/>
+        <v>154.4642125</v>
+      </c>
+      <c r="J5" s="4">
+        <v>8.5</v>
+      </c>
+      <c r="K5" s="4">
+        <v>10.4</v>
+      </c>
+      <c r="L5" s="4">
+        <v>10.7</v>
+      </c>
+      <c r="M5" s="4">
+        <v>13</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="5"/>
+        <v>155.1575</v>
+      </c>
+      <c r="O5">
+        <f t="shared" si="6"/>
+        <v>155.1765</v>
+      </c>
+      <c r="P5">
+        <f t="shared" si="7"/>
+        <v>155.17949999999999</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" si="8"/>
+        <v>155.20249999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>155.17500000000001</v>
+      </c>
+      <c r="D6">
+        <v>155.19999999999999</v>
+      </c>
+      <c r="E6">
+        <v>155.1875</v>
+      </c>
+      <c r="F6">
+        <f t="shared" si="1"/>
+        <v>155.1635</v>
+      </c>
+      <c r="G6">
+        <f t="shared" si="2"/>
+        <v>155.18650000000002</v>
+      </c>
+      <c r="H6">
+        <f t="shared" si="3"/>
+        <v>155.18650000000002</v>
+      </c>
+      <c r="I6">
+        <f t="shared" si="4"/>
+        <v>154.50160249999999</v>
+      </c>
+      <c r="J6" s="4">
+        <v>10.7</v>
+      </c>
+      <c r="K6" s="4">
+        <v>13</v>
+      </c>
+      <c r="L6" s="4">
+        <v>13.2</v>
+      </c>
+      <c r="M6" s="4">
+        <v>15.5</v>
+      </c>
+      <c r="N6">
+        <f t="shared" si="5"/>
+        <v>155.17949999999999</v>
+      </c>
+      <c r="O6">
+        <f t="shared" si="6"/>
+        <v>155.20249999999999</v>
+      </c>
+      <c r="P6">
+        <f t="shared" si="7"/>
+        <v>155.2045</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="8"/>
+        <v>155.22749999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7">
+        <v>155.19999999999999</v>
+      </c>
+      <c r="D7">
+        <v>155.22749999999999</v>
+      </c>
+      <c r="E7">
+        <v>155.21375</v>
+      </c>
+      <c r="F7">
+        <f t="shared" si="1"/>
+        <v>155.18849999999998</v>
+      </c>
+      <c r="G7">
+        <f t="shared" si="2"/>
+        <v>155.2115</v>
+      </c>
+      <c r="H7">
+        <f t="shared" si="3"/>
+        <v>155.208</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="4"/>
+        <v>154.54347749999999</v>
+      </c>
+      <c r="J7" s="4">
+        <v>13.2</v>
+      </c>
+      <c r="K7" s="4">
+        <v>15.5</v>
+      </c>
+      <c r="L7" s="4">
+        <v>16.8</v>
+      </c>
+      <c r="M7" s="4">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="N7">
+        <f t="shared" si="5"/>
+        <v>155.2045</v>
+      </c>
+      <c r="O7">
+        <f t="shared" si="6"/>
+        <v>155.22749999999999</v>
+      </c>
+      <c r="P7">
+        <f t="shared" si="7"/>
+        <v>155.2405</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="8"/>
+        <v>155.25649999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8">
+        <v>155.22749999999999</v>
+      </c>
+      <c r="D8">
+        <v>155.27000000000001</v>
+      </c>
+      <c r="E8">
+        <v>155.24875</v>
+      </c>
+      <c r="F8">
+        <f t="shared" si="1"/>
+        <v>155.21949999999998</v>
+      </c>
+      <c r="G8">
+        <f t="shared" si="2"/>
+        <v>155.2355</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="3"/>
+        <v>155.239</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="4"/>
+        <v>154.60129750000002</v>
+      </c>
+      <c r="J8" s="4">
+        <v>16.8</v>
+      </c>
+      <c r="K8" s="4">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="L8" s="4">
+        <v>19.2</v>
+      </c>
+      <c r="M8" s="4">
+        <v>21.5</v>
+      </c>
+      <c r="N8">
+        <f t="shared" si="5"/>
+        <v>155.2405</v>
+      </c>
+      <c r="O8">
+        <f t="shared" si="6"/>
+        <v>155.25649999999999</v>
+      </c>
+      <c r="P8">
+        <f t="shared" si="7"/>
+        <v>155.2645</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="8"/>
+        <v>155.28749999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2</v>
+      </c>
+      <c r="C9">
+        <v>155.27000000000001</v>
+      </c>
+      <c r="D9">
+        <v>155.29499999999999</v>
+      </c>
+      <c r="E9">
+        <v>155.2825</v>
+      </c>
+      <c r="F9">
+        <f t="shared" si="1"/>
+        <v>155.2585</v>
+      </c>
+      <c r="G9">
+        <f t="shared" si="2"/>
+        <v>155.28150000000002</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="3"/>
+        <v>155.28150000000002</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="4"/>
+        <v>154.6386775</v>
+      </c>
+      <c r="J9" s="4">
+        <v>19.2</v>
+      </c>
+      <c r="K9" s="4">
+        <v>21.5</v>
+      </c>
+      <c r="L9" s="4">
+        <v>21.7</v>
+      </c>
+      <c r="M9" s="4">
+        <v>24</v>
+      </c>
+      <c r="N9">
+        <f t="shared" si="5"/>
+        <v>155.2645</v>
+      </c>
+      <c r="O9">
+        <f t="shared" si="6"/>
+        <v>155.28749999999999</v>
+      </c>
+      <c r="P9">
+        <f t="shared" si="7"/>
+        <v>155.2895</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="8"/>
+        <v>155.3125</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
+        <v>2</v>
+      </c>
+      <c r="C10">
+        <v>155.29499999999999</v>
+      </c>
+      <c r="D10">
+        <v>155.32</v>
+      </c>
+      <c r="E10">
+        <v>155.3075</v>
+      </c>
+      <c r="F10">
+        <f t="shared" si="1"/>
+        <v>155.28349999999998</v>
+      </c>
+      <c r="G10">
+        <f t="shared" si="2"/>
+        <v>155.3065</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="3"/>
+        <v>155.28749999999999</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="4"/>
+        <v>154.66605250000001</v>
+      </c>
+      <c r="J10" s="4">
+        <v>21.7</v>
+      </c>
+      <c r="K10" s="4">
+        <v>24</v>
+      </c>
+      <c r="L10" s="4">
+        <v>26</v>
+      </c>
+      <c r="M10" s="4">
+        <v>24.5</v>
+      </c>
+      <c r="N10">
+        <f t="shared" si="5"/>
+        <v>155.2895</v>
+      </c>
+      <c r="O10">
+        <f t="shared" si="6"/>
+        <v>155.3125</v>
+      </c>
+      <c r="P10">
+        <f t="shared" si="7"/>
+        <v>155.33249999999998</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="8"/>
+        <v>155.3175</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40B097D0-02F0-D541-A913-186C44744D3E}">
-  <dimension ref="A2:I32"/>
+  <dimension ref="A2:P32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>24</v>
       </c>
@@ -1563,8 +2327,14 @@
       <c r="F4" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="G4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H4" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B5">
         <v>0</v>
       </c>
@@ -1584,7 +2354,7 @@
         <v>156.80150000000003</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B6">
         <v>26</v>
       </c>
@@ -1604,7 +2374,7 @@
         <v>156.82700000000003</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B7">
         <v>50</v>
       </c>
@@ -1624,7 +2394,7 @@
         <v>156.85100000000003</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B8">
         <v>76</v>
       </c>
@@ -1644,7 +2414,7 @@
         <v>156.875</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:16" ht="17" x14ac:dyDescent="0.2">
       <c r="B9">
         <v>110</v>
       </c>
@@ -1663,8 +2433,11 @@
         <f t="shared" si="2"/>
         <v>156.90650000000002</v>
       </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="P9" s="3">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B10">
         <v>126</v>
       </c>
@@ -1683,8 +2456,11 @@
         <f t="shared" si="2"/>
         <v>156.92700000000002</v>
       </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="P10">
+        <v>5.0999999999999996</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B11">
         <v>151</v>
       </c>
@@ -1703,8 +2479,11 @@
         <f t="shared" si="2"/>
         <v>156.95200000000003</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="P11">
+        <v>8.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B12">
         <v>176</v>
       </c>
@@ -1723,8 +2502,11 @@
         <f t="shared" si="2"/>
         <v>156.97250000000003</v>
       </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="P12">
+        <v>10.8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B13">
         <v>201</v>
       </c>
@@ -1743,8 +2525,11 @@
         <f t="shared" si="2"/>
         <v>157.00200000000001</v>
       </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="P13">
+        <v>13.3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B14">
         <v>225</v>
       </c>
@@ -1763,8 +2548,11 @@
         <f t="shared" si="2"/>
         <v>157.0265</v>
       </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="P14">
+        <v>16.399999999999999</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
       <c r="B15">
         <v>250</v>
       </c>
@@ -1783,8 +2571,21 @@
         <f t="shared" si="2"/>
         <v>157.04400000000001</v>
       </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.2">
+      <c r="P15">
+        <v>20.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="P16">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="17" spans="2:16" x14ac:dyDescent="0.2">
+      <c r="P17">
+        <v>25.9</v>
+      </c>
+    </row>
+    <row r="21" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B21" t="s">
         <v>25</v>
       </c>
@@ -1798,7 +2599,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:16" x14ac:dyDescent="0.2">
       <c r="B22">
         <v>156.77000000000001</v>
       </c>
@@ -1812,7 +2613,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H23" t="s">
         <v>14</v>
       </c>
@@ -1820,7 +2621,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H24" t="s">
         <v>15</v>
       </c>
@@ -1828,7 +2629,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="25" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H25" t="s">
         <v>16</v>
       </c>
@@ -1836,7 +2637,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="26" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H26" t="s">
         <v>17</v>
       </c>
@@ -1844,7 +2645,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="27" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H27" t="s">
         <v>18</v>
       </c>
@@ -1852,7 +2653,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H28" t="s">
         <v>19</v>
       </c>
@@ -1860,7 +2661,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="29" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H29" t="s">
         <v>20</v>
       </c>
@@ -1868,7 +2669,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="30" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H30" t="s">
         <v>21</v>
       </c>
@@ -1876,7 +2677,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="31" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H31" t="s">
         <v>22</v>
       </c>
@@ -1884,7 +2685,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="32" spans="2:9" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:16" x14ac:dyDescent="0.2">
       <c r="H32" t="s">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
add major gas isotope and ratio data from Rom; update scripts to proccess and plot
</commit_message>
<xml_diff>
--- a/data/sampling/ghg/ghg_data.xlsx
+++ b/data/sampling/ghg/ghg_data.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/ghg/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68F76373-1B2E-CE46-8727-9283B1613FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0583056-C1D5-414F-9E9D-F3850F2F3557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-7860" yWindow="-20820" windowWidth="29160" windowHeight="18980" xr2:uid="{5D78C863-DB51-414A-8C70-78F5C24BA3CE}"/>
+    <workbookView xWindow="2580" yWindow="660" windowWidth="24000" windowHeight="18980" xr2:uid="{5D78C863-DB51-414A-8C70-78F5C24BA3CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
+    <sheet name="O2N2_cuts" sheetId="4" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -60,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="75">
   <si>
     <t>section</t>
   </si>
@@ -201,6 +202,90 @@
   </si>
   <si>
     <t>bottom_right_depth</t>
+  </si>
+  <si>
+    <t>bottom_right_depth2</t>
+  </si>
+  <si>
+    <t>top_right_depth2</t>
+  </si>
+  <si>
+    <t>offset2</t>
+  </si>
+  <si>
+    <t>offset2b</t>
+  </si>
+  <si>
+    <t>d13C</t>
+  </si>
+  <si>
+    <t>section top</t>
+  </si>
+  <si>
+    <t>sample</t>
+  </si>
+  <si>
+    <t>scratch</t>
+  </si>
+  <si>
+    <t>scatch</t>
+  </si>
+  <si>
+    <t>thickness</t>
+  </si>
+  <si>
+    <t>d15N</t>
+  </si>
+  <si>
+    <t>d40Ar</t>
+  </si>
+  <si>
+    <t>d18Ograv</t>
+  </si>
+  <si>
+    <t>dO2/N2</t>
+  </si>
+  <si>
+    <t>dO2/Ar</t>
+  </si>
+  <si>
+    <t>dAr/N2</t>
+  </si>
+  <si>
+    <t>dCO2/N2</t>
+  </si>
+  <si>
+    <t>d40Ar/4</t>
+  </si>
+  <si>
+    <t>d18O_o2</t>
+  </si>
+  <si>
+    <t>d17O_2</t>
+  </si>
+  <si>
+    <t>d18O_atm</t>
+  </si>
+  <si>
+    <t>o2n2</t>
+  </si>
+  <si>
+    <t>o2n3</t>
+  </si>
+  <si>
+    <t>o2n4</t>
+  </si>
+  <si>
+    <t>o2n5</t>
+  </si>
+  <si>
+    <t>o2n6</t>
+  </si>
+  <si>
+    <t>o2n7</t>
+  </si>
+  <si>
+    <t>o2n8</t>
   </si>
 </sst>
 </file>
@@ -210,7 +295,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -236,6 +321,25 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -257,12 +361,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -597,7 +705,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC37B97-9650-DA43-B790-3970A5ED3209}">
-  <dimension ref="A1:O41"/>
+  <dimension ref="A1:AA49"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
@@ -605,7 +713,7 @@
     <col min="9" max="9" width="18.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -651,8 +759,44 @@
       <c r="O1" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="P1" t="s">
+        <v>51</v>
+      </c>
+      <c r="Q1" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="S1" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="T1" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y1" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="Z1" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="AA1" s="8" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -672,13 +816,13 @@
         <v>155.08849999999998</v>
       </c>
       <c r="G2">
-        <v>155.07749999999999</v>
+        <v>155.09249999999997</v>
       </c>
       <c r="H2">
         <v>155.10249999999999</v>
       </c>
       <c r="I2">
-        <v>155.1215</v>
+        <v>155.13649999999998</v>
       </c>
       <c r="K2">
         <v>513.39643590000003</v>
@@ -687,7 +831,7 @@
         <v>0.100997292</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -707,13 +851,13 @@
         <v>155.10249999999999</v>
       </c>
       <c r="G3">
-        <v>155.1215</v>
+        <v>155.13649999999998</v>
       </c>
       <c r="H3">
         <v>155.1275</v>
       </c>
       <c r="I3">
-        <v>155.1525</v>
+        <v>155.16749999999999</v>
       </c>
       <c r="K3">
         <v>521.20168609999996</v>
@@ -722,7 +866,7 @@
         <v>9.7894287999999996E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -742,13 +886,13 @@
         <v>155.1275</v>
       </c>
       <c r="G4">
-        <v>155.1525</v>
+        <v>155.16749999999999</v>
       </c>
       <c r="H4">
         <v>155.1575</v>
       </c>
       <c r="I4">
-        <v>155.1765</v>
+        <v>155.19149999999999</v>
       </c>
       <c r="K4">
         <v>566.79918099999998</v>
@@ -757,7 +901,7 @@
         <v>9.3101737000000004E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -777,13 +921,13 @@
         <v>155.1575</v>
       </c>
       <c r="G5">
-        <v>155.1765</v>
+        <v>155.19149999999999</v>
       </c>
       <c r="H5">
         <v>155.17949999999999</v>
       </c>
       <c r="I5">
-        <v>155.20249999999999</v>
+        <v>155.21749999999997</v>
       </c>
       <c r="K5">
         <v>575.73996339999997</v>
@@ -792,7 +936,7 @@
         <v>9.6401944000000003E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -812,13 +956,13 @@
         <v>155.17949999999999</v>
       </c>
       <c r="G6">
-        <v>155.20249999999999</v>
+        <v>155.21749999999997</v>
       </c>
       <c r="H6">
         <v>155.2045</v>
       </c>
       <c r="I6">
-        <v>155.22749999999999</v>
+        <v>155.24249999999998</v>
       </c>
       <c r="K6">
         <v>593.48608549999994</v>
@@ -827,7 +971,7 @@
         <v>0.100555226</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -847,13 +991,13 @@
         <v>155.2045</v>
       </c>
       <c r="G7">
-        <v>155.22749999999999</v>
+        <v>155.24249999999998</v>
       </c>
       <c r="H7">
         <v>155.2405</v>
       </c>
       <c r="I7">
-        <v>155.25649999999999</v>
+        <v>155.27149999999997</v>
       </c>
       <c r="K7">
         <v>618.58037349999995</v>
@@ -862,7 +1006,7 @@
         <v>9.6052947999999999E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -882,13 +1026,13 @@
         <v>155.2405</v>
       </c>
       <c r="G8">
-        <v>155.25649999999999</v>
+        <v>155.27149999999997</v>
       </c>
       <c r="H8">
         <v>155.2645</v>
       </c>
       <c r="I8">
-        <v>155.28749999999999</v>
+        <v>155.30249999999998</v>
       </c>
       <c r="K8">
         <v>627.77715360000002</v>
@@ -897,7 +1041,7 @@
         <v>9.6107177000000002E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -917,13 +1061,13 @@
         <v>155.2645</v>
       </c>
       <c r="G9">
-        <v>155.28749999999999</v>
+        <v>155.30249999999998</v>
       </c>
       <c r="H9">
         <v>155.2895</v>
       </c>
       <c r="I9">
-        <v>155.3125</v>
+        <v>155.32749999999999</v>
       </c>
       <c r="K9">
         <v>578.25503690000005</v>
@@ -932,7 +1076,7 @@
         <v>9.9159223000000005E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -952,13 +1096,13 @@
         <v>155.2895</v>
       </c>
       <c r="G10">
-        <v>155.3125</v>
+        <v>155.32749999999999</v>
       </c>
       <c r="H10">
         <v>155.33249999999998</v>
       </c>
       <c r="I10">
-        <v>155.3175</v>
+        <v>155.33249999999998</v>
       </c>
       <c r="K10">
         <v>572.04765689999999</v>
@@ -967,7 +1111,7 @@
         <v>8.5164080000000003E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -987,7 +1131,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>9</v>
       </c>
@@ -1007,7 +1151,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>9</v>
       </c>
@@ -1027,7 +1171,7 @@
         <v>799</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>9</v>
       </c>
@@ -1047,7 +1191,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>9</v>
       </c>
@@ -1067,7 +1211,7 @@
         <v>818.9</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>9</v>
       </c>
@@ -1408,7 +1552,7 @@
         <v>711.56288936566284</v>
       </c>
     </row>
-    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -1428,7 +1572,7 @@
         <v>743.06784778646261</v>
       </c>
     </row>
-    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>11</v>
       </c>
@@ -1461,7 +1605,7 @@
         <v>1.18</v>
       </c>
     </row>
-    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>11</v>
       </c>
@@ -1494,7 +1638,7 @@
         <v>2.56</v>
       </c>
     </row>
-    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>11</v>
       </c>
@@ -1527,7 +1671,7 @@
         <v>2.86</v>
       </c>
     </row>
-    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -1560,7 +1704,7 @@
         <v>1.76</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -1593,7 +1737,7 @@
         <v>2.09</v>
       </c>
     </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>11</v>
       </c>
@@ -1626,7 +1770,7 @@
         <v>1.04</v>
       </c>
     </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -1659,7 +1803,7 @@
         <v>0.97</v>
       </c>
     </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>11</v>
       </c>
@@ -1692,15 +1836,617 @@
         <v>1.33</v>
       </c>
     </row>
+    <row r="42" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>9</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C42">
+        <v>155.07249999999999</v>
+      </c>
+      <c r="D42">
+        <f>C42+0.26</f>
+        <v>155.33249999999998</v>
+      </c>
+      <c r="E42">
+        <f>(C42+D42)/2</f>
+        <v>155.20249999999999</v>
+      </c>
+      <c r="P42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>9</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C43">
+        <v>155.08949999999999</v>
+      </c>
+      <c r="D43">
+        <v>155.11449999999999</v>
+      </c>
+      <c r="E43">
+        <f>(C43+D43)/2</f>
+        <v>155.10199999999998</v>
+      </c>
+      <c r="Q43" s="7">
+        <v>6.4000000000000001E-2</v>
+      </c>
+      <c r="R43" s="7">
+        <v>0.71350000000000002</v>
+      </c>
+      <c r="S43" s="7">
+        <v>0.44869999999999999</v>
+      </c>
+      <c r="T43" s="7">
+        <v>0.4587</v>
+      </c>
+      <c r="U43" s="7">
+        <v>0.58550000000000002</v>
+      </c>
+      <c r="V43" s="7">
+        <v>-30.166899999999998</v>
+      </c>
+      <c r="W43" s="7">
+        <v>-19.9116</v>
+      </c>
+      <c r="X43" s="7">
+        <v>-10.4655</v>
+      </c>
+      <c r="Y43" s="7">
+        <v>-1.6060000000000001</v>
+      </c>
+      <c r="Z43" s="7">
+        <v>0.39750000000000002</v>
+      </c>
+      <c r="AA43" s="6">
+        <v>0.11467106000000001</v>
+      </c>
+    </row>
+    <row r="44" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>9</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C44">
+        <v>155.11449999999999</v>
+      </c>
+      <c r="D44">
+        <v>155.1395</v>
+      </c>
+      <c r="E44">
+        <f t="shared" ref="E44:E49" si="1">(C44+D44)/2</f>
+        <v>155.12700000000001</v>
+      </c>
+      <c r="Q44" s="7">
+        <v>6.3700000000000007E-2</v>
+      </c>
+      <c r="R44" s="7">
+        <v>0.67769999999999997</v>
+      </c>
+      <c r="S44" s="7">
+        <v>0.44</v>
+      </c>
+      <c r="T44" s="7">
+        <v>0.46429999999999999</v>
+      </c>
+      <c r="U44" s="7">
+        <v>0.5504</v>
+      </c>
+      <c r="V44" s="7">
+        <v>-31.575299999999999</v>
+      </c>
+      <c r="W44" s="7">
+        <v>-21.545400000000001</v>
+      </c>
+      <c r="X44" s="7">
+        <v>-10.252000000000001</v>
+      </c>
+      <c r="Y44" s="7">
+        <v>-2.0933000000000002</v>
+      </c>
+      <c r="Z44" s="7">
+        <v>0.34239999999999998</v>
+      </c>
+      <c r="AA44" s="6">
+        <v>0.11608642</v>
+      </c>
+    </row>
+    <row r="45" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>9</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="C45">
+        <v>155.1395</v>
+      </c>
+      <c r="D45">
+        <v>155.16249999999999</v>
+      </c>
+      <c r="E45">
+        <f t="shared" si="1"/>
+        <v>155.15100000000001</v>
+      </c>
+      <c r="Q45" s="7">
+        <v>6.4899999999999999E-2</v>
+      </c>
+      <c r="R45" s="7">
+        <v>0.64370000000000005</v>
+      </c>
+      <c r="S45" s="7">
+        <v>0.44030000000000002</v>
+      </c>
+      <c r="T45" s="7">
+        <v>0.4254</v>
+      </c>
+      <c r="U45" s="7">
+        <v>0.51390000000000002</v>
+      </c>
+      <c r="V45" s="7">
+        <v>-27.553699999999999</v>
+      </c>
+      <c r="W45" s="7">
+        <v>-19.6982</v>
+      </c>
+      <c r="X45" s="7">
+        <v>-8.0136000000000003</v>
+      </c>
+      <c r="Y45" s="7">
+        <v>-1.6769000000000001</v>
+      </c>
+      <c r="Z45" s="7">
+        <v>0.31919999999999998</v>
+      </c>
+      <c r="AA45" s="6">
+        <v>0.1063529</v>
+      </c>
+    </row>
+    <row r="46" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>9</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C46">
+        <v>155.17749999999998</v>
+      </c>
+      <c r="D46">
+        <v>155.20749999999998</v>
+      </c>
+      <c r="E46">
+        <f t="shared" si="1"/>
+        <v>155.1925</v>
+      </c>
+      <c r="Q46" s="7">
+        <v>6.0600000000000001E-2</v>
+      </c>
+      <c r="R46" s="7">
+        <v>0.62649999999999995</v>
+      </c>
+      <c r="S46" s="7">
+        <v>0.4178</v>
+      </c>
+      <c r="T46" s="7">
+        <v>0.45779999999999998</v>
+      </c>
+      <c r="U46" s="7">
+        <v>0.50529999999999997</v>
+      </c>
+      <c r="V46" s="7">
+        <v>-34.302700000000002</v>
+      </c>
+      <c r="W46" s="7">
+        <v>-23.440200000000001</v>
+      </c>
+      <c r="X46" s="7">
+        <v>-11.122999999999999</v>
+      </c>
+      <c r="Y46" s="7">
+        <v>-3.5758999999999999</v>
+      </c>
+      <c r="Z46" s="7">
+        <v>0.27789999999999998</v>
+      </c>
+      <c r="AA46" s="6">
+        <v>0.11445104</v>
+      </c>
+    </row>
+    <row r="47" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>9</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C47">
+        <v>155.20749999999998</v>
+      </c>
+      <c r="D47">
+        <v>155.23650000000001</v>
+      </c>
+      <c r="E47">
+        <f t="shared" si="1"/>
+        <v>155.22199999999998</v>
+      </c>
+      <c r="Q47" s="7">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="R47" s="7">
+        <v>0.60780000000000001</v>
+      </c>
+      <c r="S47" s="7">
+        <v>0.42909999999999998</v>
+      </c>
+      <c r="T47" s="7">
+        <v>0.45429999999999998</v>
+      </c>
+      <c r="U47" s="7">
+        <v>0.49580000000000002</v>
+      </c>
+      <c r="V47" s="7">
+        <v>-31.6357</v>
+      </c>
+      <c r="W47" s="7">
+        <v>-22.866900000000001</v>
+      </c>
+      <c r="X47" s="7">
+        <v>-8.9747000000000003</v>
+      </c>
+      <c r="Y47" s="7">
+        <v>-3.0928</v>
+      </c>
+      <c r="Z47" s="7">
+        <v>0.26619999999999999</v>
+      </c>
+      <c r="AA47" s="6">
+        <v>0.11358240999999999</v>
+      </c>
+    </row>
+    <row r="48" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>9</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C48">
+        <v>155.26349999999999</v>
+      </c>
+      <c r="D48">
+        <v>155.29249999999999</v>
+      </c>
+      <c r="E48">
+        <f t="shared" si="1"/>
+        <v>155.27799999999999</v>
+      </c>
+      <c r="Q48" s="7">
+        <v>5.7599999999999998E-2</v>
+      </c>
+      <c r="R48" s="7">
+        <v>0.64270000000000005</v>
+      </c>
+      <c r="S48" s="7">
+        <v>0.44850000000000001</v>
+      </c>
+      <c r="T48" s="7">
+        <v>0.4995</v>
+      </c>
+      <c r="U48" s="7">
+        <v>0.52759999999999996</v>
+      </c>
+      <c r="V48" s="7">
+        <v>-34.093899999999998</v>
+      </c>
+      <c r="W48" s="7">
+        <v>-23.976800000000001</v>
+      </c>
+      <c r="X48" s="7">
+        <v>-10.365500000000001</v>
+      </c>
+      <c r="Y48" s="7">
+        <v>-5.0655000000000001</v>
+      </c>
+      <c r="Z48" s="7">
+        <v>0.29049999999999998</v>
+      </c>
+      <c r="AA48" s="6">
+        <v>0.12486915</v>
+      </c>
+    </row>
+    <row r="49" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>9</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49">
+        <v>155.29249999999999</v>
+      </c>
+      <c r="D49">
+        <v>155.32249999999999</v>
+      </c>
+      <c r="E49">
+        <f t="shared" si="1"/>
+        <v>155.3075</v>
+      </c>
+      <c r="Q49" s="7">
+        <v>6.6799999999999998E-2</v>
+      </c>
+      <c r="R49" s="7">
+        <v>0.64890000000000003</v>
+      </c>
+      <c r="S49" s="7">
+        <v>0.45069999999999999</v>
+      </c>
+      <c r="T49" s="7">
+        <v>0.53210000000000002</v>
+      </c>
+      <c r="U49" s="7">
+        <v>0.51539999999999997</v>
+      </c>
+      <c r="V49" s="7">
+        <v>-34.400799999999997</v>
+      </c>
+      <c r="W49" s="7">
+        <v>-24.283000000000001</v>
+      </c>
+      <c r="X49" s="7">
+        <v>-10.369899999999999</v>
+      </c>
+      <c r="Y49" s="7">
+        <v>-5.5232999999999999</v>
+      </c>
+      <c r="Z49" s="7">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AA49" s="6">
+        <v>0.13301735000000001</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FC3C9996-0E34-9A42-84FB-8FC0301D0367}">
+  <dimension ref="A4:I24"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="B4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C4" s="6">
+        <v>155.07249999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="H5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="E6" s="5">
+        <v>155.08199999999999</v>
+      </c>
+      <c r="F6" s="5">
+        <v>155.107</v>
+      </c>
+      <c r="H6">
+        <f>E6-155.065+155.0725</f>
+        <v>155.08949999999999</v>
+      </c>
+      <c r="I6">
+        <f>F6-155.065+155.0725</f>
+        <v>155.11449999999999</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E7" s="5">
+        <v>155.107</v>
+      </c>
+      <c r="F7" s="5">
+        <v>155.13200000000001</v>
+      </c>
+      <c r="H7">
+        <f t="shared" ref="H7:I12" si="0">E7-155.065+155.0725</f>
+        <v>155.11449999999999</v>
+      </c>
+      <c r="I7">
+        <f t="shared" si="0"/>
+        <v>155.1395</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E8" s="5">
+        <v>155.13200000000001</v>
+      </c>
+      <c r="F8" s="5">
+        <v>155.155</v>
+      </c>
+      <c r="H8">
+        <f t="shared" si="0"/>
+        <v>155.1395</v>
+      </c>
+      <c r="I8">
+        <f t="shared" si="0"/>
+        <v>155.16249999999999</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9">
+        <v>1.7</v>
+      </c>
+      <c r="E9" s="5">
+        <v>155.16999999999999</v>
+      </c>
+      <c r="F9" s="5">
+        <v>155.19999999999999</v>
+      </c>
+      <c r="H9">
+        <f t="shared" si="0"/>
+        <v>155.17749999999998</v>
+      </c>
+      <c r="I9">
+        <f t="shared" si="0"/>
+        <v>155.20749999999998</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A10">
+        <v>2</v>
+      </c>
+      <c r="B10">
+        <v>2.5</v>
+      </c>
+      <c r="E10" s="5">
+        <v>155.19999999999999</v>
+      </c>
+      <c r="F10" s="5">
+        <v>155.22900000000001</v>
+      </c>
+      <c r="H10">
+        <f t="shared" si="0"/>
+        <v>155.20749999999998</v>
+      </c>
+      <c r="I10">
+        <f t="shared" si="0"/>
+        <v>155.23650000000001</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A11">
+        <v>3</v>
+      </c>
+      <c r="B11">
+        <v>2.5</v>
+      </c>
+      <c r="E11" s="5">
+        <v>155.256</v>
+      </c>
+      <c r="F11" s="5">
+        <v>155.285</v>
+      </c>
+      <c r="H11">
+        <f t="shared" si="0"/>
+        <v>155.26349999999999</v>
+      </c>
+      <c r="I11">
+        <f t="shared" si="0"/>
+        <v>155.29249999999999</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12">
+        <v>1.5</v>
+      </c>
+      <c r="E12" s="5">
+        <v>155.285</v>
+      </c>
+      <c r="F12" s="5">
+        <v>155.315</v>
+      </c>
+      <c r="H12">
+        <f t="shared" si="0"/>
+        <v>155.29249999999999</v>
+      </c>
+      <c r="I12">
+        <f t="shared" si="0"/>
+        <v>155.32249999999999</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A13">
+        <v>4</v>
+      </c>
+      <c r="B13">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A14">
+        <v>5</v>
+      </c>
+      <c r="B14">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>6</v>
+      </c>
+      <c r="B16">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>7</v>
+      </c>
+      <c r="B17">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="B24">
+        <f>SUM(B9:B17)</f>
+        <v>22.7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75A36881-0611-A543-91F5-CA8955EF1326}">
-  <dimension ref="A1:Q10"/>
+  <dimension ref="A1:V13"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="20.6640625" customWidth="1"/>
@@ -1709,7 +2455,7 @@
     <col min="9" max="9" width="28.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1749,8 +2495,23 @@
       <c r="Q1" t="s">
         <v>46</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R1" t="s">
+        <v>26</v>
+      </c>
+      <c r="S1" t="s">
+        <v>48</v>
+      </c>
+      <c r="T1" t="s">
+        <v>47</v>
+      </c>
+      <c r="U1" t="s">
+        <v>49</v>
+      </c>
+      <c r="V1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -1799,7 +2560,7 @@
         <v>155.08849999999998</v>
       </c>
       <c r="O2">
-        <f t="shared" ref="O2:R2" si="0">$C$2+K2/100</f>
+        <f t="shared" ref="O2:Q2" si="0">$C$2+K2/100</f>
         <v>155.07749999999999</v>
       </c>
       <c r="P2">
@@ -1810,8 +2571,28 @@
         <f t="shared" si="0"/>
         <v>155.1215</v>
       </c>
-    </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R2">
+        <f>N2-O2</f>
+        <v>1.099999999999568E-2</v>
+      </c>
+      <c r="S2">
+        <f>O2+0.015</f>
+        <v>155.09249999999997</v>
+      </c>
+      <c r="T2">
+        <f>Q2+0.015</f>
+        <v>155.13649999999998</v>
+      </c>
+      <c r="U2">
+        <f>N2-S2</f>
+        <v>-3.9999999999906777E-3</v>
+      </c>
+      <c r="V2">
+        <f>P2-T2</f>
+        <v>-3.3999999999991815E-2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -1871,8 +2652,28 @@
         <f t="shared" ref="Q3:Q10" si="8">$C$2+M3/100</f>
         <v>155.1525</v>
       </c>
-    </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R3">
+        <f t="shared" ref="R3:R10" si="9">N3-O3</f>
+        <v>-1.9000000000005457E-2</v>
+      </c>
+      <c r="S3">
+        <f t="shared" ref="S3:S10" si="10">O3+0.015</f>
+        <v>155.13649999999998</v>
+      </c>
+      <c r="T3">
+        <f t="shared" ref="T3:T10" si="11">Q3+0.015</f>
+        <v>155.16749999999999</v>
+      </c>
+      <c r="U3">
+        <f t="shared" ref="U3:U10" si="12">N3-S3</f>
+        <v>-3.3999999999991815E-2</v>
+      </c>
+      <c r="V3">
+        <f t="shared" ref="V3:V10" si="13">P3-T3</f>
+        <v>-3.9999999999992042E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -1932,8 +2733,28 @@
         <f t="shared" si="8"/>
         <v>155.1765</v>
       </c>
-    </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R4">
+        <f t="shared" si="9"/>
+        <v>-2.5000000000005684E-2</v>
+      </c>
+      <c r="S4">
+        <f t="shared" si="10"/>
+        <v>155.16749999999999</v>
+      </c>
+      <c r="T4">
+        <f t="shared" si="11"/>
+        <v>155.19149999999999</v>
+      </c>
+      <c r="U4">
+        <f t="shared" si="12"/>
+        <v>-3.9999999999992042E-2</v>
+      </c>
+      <c r="V4">
+        <f t="shared" si="13"/>
+        <v>-3.3999999999991815E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -1993,8 +2814,28 @@
         <f t="shared" si="8"/>
         <v>155.20249999999999</v>
       </c>
-    </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R5">
+        <f t="shared" si="9"/>
+        <v>-1.9000000000005457E-2</v>
+      </c>
+      <c r="S5">
+        <f t="shared" si="10"/>
+        <v>155.19149999999999</v>
+      </c>
+      <c r="T5">
+        <f t="shared" si="11"/>
+        <v>155.21749999999997</v>
+      </c>
+      <c r="U5">
+        <f t="shared" si="12"/>
+        <v>-3.3999999999991815E-2</v>
+      </c>
+      <c r="V5">
+        <f t="shared" si="13"/>
+        <v>-3.7999999999982492E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -2054,8 +2895,28 @@
         <f t="shared" si="8"/>
         <v>155.22749999999999</v>
       </c>
-    </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R6">
+        <f t="shared" si="9"/>
+        <v>-2.2999999999996135E-2</v>
+      </c>
+      <c r="S6">
+        <f t="shared" si="10"/>
+        <v>155.21749999999997</v>
+      </c>
+      <c r="T6">
+        <f t="shared" si="11"/>
+        <v>155.24249999999998</v>
+      </c>
+      <c r="U6">
+        <f t="shared" si="12"/>
+        <v>-3.7999999999982492E-2</v>
+      </c>
+      <c r="V6">
+        <f t="shared" si="13"/>
+        <v>-3.7999999999982492E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -2115,8 +2976,28 @@
         <f t="shared" si="8"/>
         <v>155.25649999999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R7">
+        <f t="shared" si="9"/>
+        <v>-2.2999999999996135E-2</v>
+      </c>
+      <c r="S7">
+        <f t="shared" si="10"/>
+        <v>155.24249999999998</v>
+      </c>
+      <c r="T7">
+        <f t="shared" si="11"/>
+        <v>155.27149999999997</v>
+      </c>
+      <c r="U7">
+        <f t="shared" si="12"/>
+        <v>-3.7999999999982492E-2</v>
+      </c>
+      <c r="V7">
+        <f t="shared" si="13"/>
+        <v>-3.099999999997749E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -2176,8 +3057,28 @@
         <f t="shared" si="8"/>
         <v>155.28749999999999</v>
       </c>
-    </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R8">
+        <f t="shared" si="9"/>
+        <v>-1.5999999999991132E-2</v>
+      </c>
+      <c r="S8">
+        <f t="shared" si="10"/>
+        <v>155.27149999999997</v>
+      </c>
+      <c r="T8">
+        <f t="shared" si="11"/>
+        <v>155.30249999999998</v>
+      </c>
+      <c r="U8">
+        <f t="shared" si="12"/>
+        <v>-3.099999999997749E-2</v>
+      </c>
+      <c r="V8">
+        <f t="shared" si="13"/>
+        <v>-3.7999999999982492E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -2237,8 +3138,28 @@
         <f t="shared" si="8"/>
         <v>155.3125</v>
       </c>
-    </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="R9">
+        <f t="shared" si="9"/>
+        <v>-2.2999999999996135E-2</v>
+      </c>
+      <c r="S9">
+        <f t="shared" si="10"/>
+        <v>155.30249999999998</v>
+      </c>
+      <c r="T9">
+        <f t="shared" si="11"/>
+        <v>155.32749999999999</v>
+      </c>
+      <c r="U9">
+        <f t="shared" si="12"/>
+        <v>-3.7999999999982492E-2</v>
+      </c>
+      <c r="V9">
+        <f t="shared" si="13"/>
+        <v>-3.7999999999982492E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -2297,6 +3218,32 @@
       <c r="Q10">
         <f t="shared" si="8"/>
         <v>155.3175</v>
+      </c>
+      <c r="R10">
+        <f t="shared" si="9"/>
+        <v>-2.2999999999996135E-2</v>
+      </c>
+      <c r="S10">
+        <f t="shared" si="10"/>
+        <v>155.32749999999999</v>
+      </c>
+      <c r="T10">
+        <f t="shared" si="11"/>
+        <v>155.33249999999998</v>
+      </c>
+      <c r="U10">
+        <f t="shared" si="12"/>
+        <v>-3.7999999999982492E-2</v>
+      </c>
+      <c r="V10">
+        <f t="shared" si="13"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:22" x14ac:dyDescent="0.2">
+      <c r="U13">
+        <f>0.53-0.38</f>
+        <v>0.15000000000000002</v>
       </c>
     </row>
   </sheetData>
@@ -2304,7 +3251,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{40B097D0-02F0-D541-A913-186C44744D3E}">
   <dimension ref="A2:P32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
finetune implimentation of major gas data. Fix units, spacing on graph, etc
</commit_message>
<xml_diff>
--- a/data/sampling/ghg/ghg_data.xlsx
+++ b/data/sampling/ghg/ghg_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Liam/Desktop/UW/paper2/github/data/sampling/ghg/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0583056-C1D5-414F-9E9D-F3850F2F3557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97D2F572-5654-B24D-BBBB-71B49B228A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2580" yWindow="660" windowWidth="24000" windowHeight="18980" xr2:uid="{5D78C863-DB51-414A-8C70-78F5C24BA3CE}"/>
+    <workbookView xWindow="1460" yWindow="-22120" windowWidth="24000" windowHeight="18980" xr2:uid="{5D78C863-DB51-414A-8C70-78F5C24BA3CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="74">
   <si>
     <t>section</t>
   </si>
@@ -253,9 +253,6 @@
   </si>
   <si>
     <t>dCO2/N2</t>
-  </si>
-  <si>
-    <t>d40Ar/4</t>
   </si>
   <si>
     <t>d18O_o2</t>
@@ -361,7 +358,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -369,7 +366,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -762,39 +758,37 @@
       <c r="P1" t="s">
         <v>51</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="Q1" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="S1" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="T1" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="U1" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="V1" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="W1" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="X1" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="Y1" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="Z1" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="T1" s="8" t="s">
-        <v>58</v>
-      </c>
-      <c r="U1" s="8" t="s">
-        <v>59</v>
-      </c>
-      <c r="V1" s="8" t="s">
-        <v>60</v>
-      </c>
-      <c r="W1" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="X1" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="Y1" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="Z1" s="8" t="s">
-        <v>67</v>
-      </c>
-      <c r="AA1" s="8" t="s">
-        <v>64</v>
-      </c>
+      <c r="AA1" s="7"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1863,7 +1857,7 @@
         <v>9</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C43">
         <v>155.08949999999999</v>
@@ -1875,46 +1869,44 @@
         <f>(C43+D43)/2</f>
         <v>155.10199999999998</v>
       </c>
-      <c r="Q43" s="7">
+      <c r="Q43">
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="R43" s="7">
-        <v>0.71350000000000002</v>
-      </c>
-      <c r="S43" s="7">
+      <c r="R43">
+        <v>0.71440000000000003</v>
+      </c>
+      <c r="S43">
         <v>0.44869999999999999</v>
       </c>
-      <c r="T43" s="7">
+      <c r="T43">
         <v>0.4587</v>
       </c>
-      <c r="U43" s="7">
-        <v>0.58550000000000002</v>
-      </c>
-      <c r="V43" s="7">
+      <c r="U43">
+        <v>0.58650000000000002</v>
+      </c>
+      <c r="V43">
         <v>-30.166899999999998</v>
       </c>
-      <c r="W43" s="7">
+      <c r="W43">
         <v>-19.9116</v>
       </c>
-      <c r="X43" s="7">
-        <v>-10.4655</v>
-      </c>
-      <c r="Y43" s="7">
+      <c r="X43">
+        <v>-9.7906999999999993</v>
+      </c>
+      <c r="Y43">
         <v>-1.6060000000000001</v>
       </c>
-      <c r="Z43" s="7">
-        <v>0.39750000000000002</v>
-      </c>
-      <c r="AA43" s="6">
-        <v>0.11467106000000001</v>
-      </c>
+      <c r="Z43">
+        <v>0.3881</v>
+      </c>
+      <c r="AA43" s="6"/>
     </row>
     <row r="44" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>9</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C44">
         <v>155.11449999999999</v>
@@ -1926,46 +1918,44 @@
         <f t="shared" ref="E44:E49" si="1">(C44+D44)/2</f>
         <v>155.12700000000001</v>
       </c>
-      <c r="Q44" s="7">
-        <v>6.3700000000000007E-2</v>
-      </c>
-      <c r="R44" s="7">
-        <v>0.67769999999999997</v>
-      </c>
-      <c r="S44" s="7">
+      <c r="Q44">
+        <v>6.3600000000000004E-2</v>
+      </c>
+      <c r="R44">
+        <v>0.67859999999999998</v>
+      </c>
+      <c r="S44">
         <v>0.44</v>
       </c>
-      <c r="T44" s="7">
+      <c r="T44">
         <v>0.46429999999999999</v>
       </c>
-      <c r="U44" s="7">
-        <v>0.5504</v>
-      </c>
-      <c r="V44" s="7">
+      <c r="U44">
+        <v>0.5514</v>
+      </c>
+      <c r="V44">
         <v>-31.575299999999999</v>
       </c>
-      <c r="W44" s="7">
+      <c r="W44">
         <v>-21.545400000000001</v>
       </c>
-      <c r="X44" s="7">
-        <v>-10.252000000000001</v>
-      </c>
-      <c r="Y44" s="7">
+      <c r="X44">
+        <v>-9.5457999999999998</v>
+      </c>
+      <c r="Y44">
         <v>-2.0933000000000002</v>
       </c>
-      <c r="Z44" s="7">
-        <v>0.34239999999999998</v>
-      </c>
-      <c r="AA44" s="6">
-        <v>0.11608642</v>
-      </c>
+      <c r="Z44">
+        <v>0.33239999999999997</v>
+      </c>
+      <c r="AA44" s="6"/>
     </row>
     <row r="45" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>9</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C45">
         <v>155.1395</v>
@@ -1977,46 +1967,44 @@
         <f t="shared" si="1"/>
         <v>155.15100000000001</v>
       </c>
-      <c r="Q45" s="7">
+      <c r="Q45">
         <v>6.4899999999999999E-2</v>
       </c>
-      <c r="R45" s="7">
-        <v>0.64370000000000005</v>
-      </c>
-      <c r="S45" s="7">
+      <c r="R45">
+        <v>0.64449999999999996</v>
+      </c>
+      <c r="S45">
         <v>0.44030000000000002</v>
       </c>
-      <c r="T45" s="7">
+      <c r="T45">
         <v>0.4254</v>
       </c>
-      <c r="U45" s="7">
-        <v>0.51390000000000002</v>
-      </c>
-      <c r="V45" s="7">
+      <c r="U45">
+        <v>0.51480000000000004</v>
+      </c>
+      <c r="V45">
         <v>-27.553699999999999</v>
       </c>
-      <c r="W45" s="7">
+      <c r="W45">
         <v>-19.6982</v>
       </c>
-      <c r="X45" s="7">
-        <v>-8.0136000000000003</v>
-      </c>
-      <c r="Y45" s="7">
+      <c r="X45">
+        <v>-7.3973000000000004</v>
+      </c>
+      <c r="Y45">
         <v>-1.6769000000000001</v>
       </c>
-      <c r="Z45" s="7">
-        <v>0.31919999999999998</v>
-      </c>
-      <c r="AA45" s="6">
-        <v>0.1063529</v>
-      </c>
+      <c r="Z45">
+        <v>0.3105</v>
+      </c>
+      <c r="AA45" s="6"/>
     </row>
     <row r="46" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>9</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C46">
         <v>155.17749999999998</v>
@@ -2028,46 +2016,44 @@
         <f t="shared" si="1"/>
         <v>155.1925</v>
       </c>
-      <c r="Q46" s="7">
-        <v>6.0600000000000001E-2</v>
-      </c>
-      <c r="R46" s="7">
-        <v>0.62649999999999995</v>
-      </c>
-      <c r="S46" s="7">
+      <c r="Q46">
+        <v>6.0499999999999998E-2</v>
+      </c>
+      <c r="R46">
+        <v>0.62739999999999996</v>
+      </c>
+      <c r="S46">
         <v>0.4178</v>
       </c>
-      <c r="T46" s="7">
+      <c r="T46">
         <v>0.45779999999999998</v>
       </c>
-      <c r="U46" s="7">
-        <v>0.50529999999999997</v>
-      </c>
-      <c r="V46" s="7">
+      <c r="U46">
+        <v>0.50629999999999997</v>
+      </c>
+      <c r="V46">
         <v>-34.302700000000002</v>
       </c>
-      <c r="W46" s="7">
+      <c r="W46">
         <v>-23.440200000000001</v>
       </c>
-      <c r="X46" s="7">
-        <v>-11.122999999999999</v>
-      </c>
-      <c r="Y46" s="7">
+      <c r="X46">
+        <v>-10.355700000000001</v>
+      </c>
+      <c r="Y46">
         <v>-3.5758999999999999</v>
       </c>
-      <c r="Z46" s="7">
-        <v>0.27789999999999998</v>
-      </c>
-      <c r="AA46" s="6">
-        <v>0.11445104</v>
-      </c>
+      <c r="Z46">
+        <v>0.26700000000000002</v>
+      </c>
+      <c r="AA46" s="6"/>
     </row>
     <row r="47" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>9</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C47">
         <v>155.20749999999998</v>
@@ -2079,46 +2065,44 @@
         <f t="shared" si="1"/>
         <v>155.22199999999998</v>
       </c>
-      <c r="Q47" s="7">
-        <v>5.6000000000000001E-2</v>
-      </c>
-      <c r="R47" s="7">
-        <v>0.60780000000000001</v>
-      </c>
-      <c r="S47" s="7">
+      <c r="Q47">
+        <v>5.5899999999999998E-2</v>
+      </c>
+      <c r="R47">
+        <v>0.60870000000000002</v>
+      </c>
+      <c r="S47">
         <v>0.42909999999999998</v>
       </c>
-      <c r="T47" s="7">
+      <c r="T47">
         <v>0.45429999999999998</v>
       </c>
-      <c r="U47" s="7">
-        <v>0.49580000000000002</v>
-      </c>
-      <c r="V47" s="7">
+      <c r="U47">
+        <v>0.49680000000000002</v>
+      </c>
+      <c r="V47">
         <v>-31.6357</v>
       </c>
-      <c r="W47" s="7">
+      <c r="W47">
         <v>-22.866900000000001</v>
       </c>
-      <c r="X47" s="7">
-        <v>-8.9747000000000003</v>
-      </c>
-      <c r="Y47" s="7">
+      <c r="X47">
+        <v>-8.2670999999999992</v>
+      </c>
+      <c r="Y47">
         <v>-3.0928</v>
       </c>
-      <c r="Z47" s="7">
-        <v>0.26619999999999999</v>
-      </c>
-      <c r="AA47" s="6">
-        <v>0.11358240999999999</v>
-      </c>
+      <c r="Z47">
+        <v>0.25619999999999998</v>
+      </c>
+      <c r="AA47" s="6"/>
     </row>
     <row r="48" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>9</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C48">
         <v>155.26349999999999</v>
@@ -2130,46 +2114,44 @@
         <f t="shared" si="1"/>
         <v>155.27799999999999</v>
       </c>
-      <c r="Q48" s="7">
-        <v>5.7599999999999998E-2</v>
-      </c>
-      <c r="R48" s="7">
-        <v>0.64270000000000005</v>
-      </c>
-      <c r="S48" s="7">
+      <c r="Q48">
+        <v>5.7500000000000002E-2</v>
+      </c>
+      <c r="R48">
+        <v>0.64359999999999995</v>
+      </c>
+      <c r="S48">
         <v>0.44850000000000001</v>
       </c>
-      <c r="T48" s="7">
+      <c r="T48">
         <v>0.4995</v>
       </c>
-      <c r="U48" s="7">
-        <v>0.52759999999999996</v>
-      </c>
-      <c r="V48" s="7">
+      <c r="U48">
+        <v>0.52859999999999996</v>
+      </c>
+      <c r="V48">
         <v>-34.093899999999998</v>
       </c>
-      <c r="W48" s="7">
+      <c r="W48">
         <v>-23.976800000000001</v>
       </c>
-      <c r="X48" s="7">
-        <v>-10.365500000000001</v>
-      </c>
-      <c r="Y48" s="7">
+      <c r="X48">
+        <v>-9.6029</v>
+      </c>
+      <c r="Y48">
         <v>-5.0655000000000001</v>
       </c>
-      <c r="Z48" s="7">
-        <v>0.29049999999999998</v>
-      </c>
-      <c r="AA48" s="6">
-        <v>0.12486915</v>
-      </c>
+      <c r="Z48">
+        <v>0.2797</v>
+      </c>
+      <c r="AA48" s="6"/>
     </row>
     <row r="49" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>9</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C49">
         <v>155.29249999999999</v>
@@ -2181,39 +2163,37 @@
         <f t="shared" si="1"/>
         <v>155.3075</v>
       </c>
-      <c r="Q49" s="7">
-        <v>6.6799999999999998E-2</v>
-      </c>
-      <c r="R49" s="7">
-        <v>0.64890000000000003</v>
-      </c>
-      <c r="S49" s="7">
+      <c r="Q49">
+        <v>6.6699999999999995E-2</v>
+      </c>
+      <c r="R49">
+        <v>0.64970000000000006</v>
+      </c>
+      <c r="S49">
         <v>0.45069999999999999</v>
       </c>
-      <c r="T49" s="7">
+      <c r="T49">
         <v>0.53210000000000002</v>
       </c>
-      <c r="U49" s="7">
-        <v>0.51539999999999997</v>
-      </c>
-      <c r="V49" s="7">
+      <c r="U49">
+        <v>0.51629999999999998</v>
+      </c>
+      <c r="V49">
         <v>-34.400799999999997</v>
       </c>
-      <c r="W49" s="7">
+      <c r="W49">
         <v>-24.283000000000001</v>
       </c>
-      <c r="X49" s="7">
-        <v>-10.369899999999999</v>
-      </c>
-      <c r="Y49" s="7">
+      <c r="X49">
+        <v>-9.6004000000000005</v>
+      </c>
+      <c r="Y49">
         <v>-5.5232999999999999</v>
       </c>
-      <c r="Z49" s="7">
-        <v>0.27600000000000002</v>
-      </c>
-      <c r="AA49" s="6">
-        <v>0.13301735000000001</v>
-      </c>
+      <c r="Z49">
+        <v>0.26500000000000001</v>
+      </c>
+      <c r="AA49" s="6"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>